<commit_message>
feat: update README for JOH submission, add paper figure scripts and SA tools
- Rewrite README with data requirements, figure reproduction table, runtime info
- Fix terminology: no-adaptation (not worst-case), homeownership status (not tenure)
- Add .ai/ to .gitignore
- Add all plot_*.py scripts for paper figure generation
- Add SA scripts (ratio threshold, decision threshold sweeps)
- Add Monte Carlo runner and validation scripts
- Update calibration pipeline outputs (phase 1-3)
- Update config and model files for owner/renter naming

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/calibration/phase2_bayesian_regression/owner_group/BP/BP_prob_metrics.xlsx
+++ b/calibration/phase2_bayesian_regression/owner_group/BP/BP_prob_metrics.xlsx
@@ -112,47 +112,55 @@
     <t>none</t>
   </si>
   <si>
-    <t>platt</t>
-  </si>
-  <si>
-    <t>{'coef': 0.03963760888167843, 'intercept': -1.4455323105842037, 'C': 1.0}</t>
-  </si>
-  <si>
-    <t>{'coef': 0.7900712707148305, 'intercept': -0.7021989247963228, 'C': 1.0}</t>
-  </si>
-  <si>
-    <t>[0.18420173 0.18079808 0.18546588 0.18315869 0.18584452 0.18284976
- 0.18671377 0.18831177 0.18517635 0.18375125 0.1859561  0.18360186
- 0.18294886 0.18696892 0.18662126 0.18907266 0.18478278 0.19246253
- 0.18664079 0.18534227 0.18761918 0.1887396  0.18556976 0.18427059
- 0.18748717 0.18549627 0.18598374 0.18304793 0.18598374 0.19091816
- 0.18111339 0.18341893 0.19075793 0.1864396  0.19636101 0.18648439
- 0.18514064 0.18534382 0.18469471 0.19324698 0.18686675 0.18400924
- 0.18527248 0.18835604 0.18410365 0.18362524 0.18544138 0.18585877
- 0.1872652  0.18423151 0.18168316 0.18533867 0.18481395 0.1788606
- 0.18997328 0.18602487 0.18825282 0.18550011 0.18342897 0.18765809
- 0.18621149 0.18399193 0.18742753 0.18742786 0.18173976 0.18719723
- 0.18838428 0.18260313 0.18717331 0.18933679 0.1897286  0.18381825
- 0.1847827  0.18631284 0.18453571 0.18511948 0.18569352 0.18969666
- 0.18613147 0.18337648 0.19006006 0.19218625 0.18365865 0.18489475
- 0.18503985 0.18526915]</t>
-  </si>
-  <si>
-    <t>[0.2238983  0.16459158 0.20655179 0.23110875 0.35359827 0.16370285
- 0.41651124 0.28561357 0.2216752  0.2003888  0.2216752  0.33326632
- 0.21581359 0.17753915 0.5425771  0.25937235 0.4298338  0.22804262
- 0.2102709  0.21523574 0.12200453 0.3274632  0.1396023  0.20866434
- 0.25297487 0.24092357 0.3412075  0.14412305 0.15722331 0.19252887
- 0.2581344  0.27538097 0.23690069 0.2786522  0.10199859 0.17685169
- 0.2265992  0.31921095 0.15668693 0.2209494  0.23934165 0.24811284
- 0.29801023 0.44859466 0.22999577 0.15432297 0.14619893 0.21231426
- 0.2620764  0.1665556  0.21523574 0.35269707 0.29443982 0.3689746
- 0.37131977 0.20374984 0.339962   0.10611171 0.34288597 0.23458244
- 0.2805127  0.37049815 0.17062245 0.24894316 0.14586137 0.37136984
- 0.19579278 0.25075734 0.29588062 0.18297979 0.16459158 0.36824876
- 0.24957453 0.11784308 0.26674834 0.1924749  0.19198774 0.23635535
- 0.19619164 0.19035955 0.2180786  0.2652047  0.25553417 0.28316092
- 0.13000596 0.38551047 0.08612181]</t>
+    <t>beta</t>
+  </si>
+  <si>
+    <t>{'a': -2.5864355866334954, 'b': -6.84091872913221, 'c': -7.254707784149799}</t>
+  </si>
+  <si>
+    <t>{'a': -2.45337502211736, 'b': -7.207566547518475, 'c': -7.056096722715588}</t>
+  </si>
+  <si>
+    <t>[0.15336176 0.22343905 0.50447    0.1705625  0.15604755 0.40016292
+ 0.19729336 0.15515122 0.15887112 0.25595881 0.15309621 0.15275213
+ 0.2361128  0.18700737 0.20376555 0.17809522 0.1584144  0.1560963
+ 0.19065361 0.21646522 0.21393747 0.21806864 0.17305625 0.62188752
+ 0.30652184 0.15572452 0.15394913 0.32734331 0.15397022 0.26286507
+ 0.17982768 0.17233776 0.16264577 0.18531928 0.1734891  0.16038417
+ 0.15250046 0.54286639 0.16727515 0.1544704  0.19954494 0.80673093
+ 0.15243321 0.17897647 0.2045184  0.16264577 0.15255277 0.19918089
+ 0.19141032 0.18736531 0.19099323 0.16515707 0.18502368 0.1524315
+ 0.15320606 0.17356529 0.20234398 0.34195994 0.21976559 0.19225808
+ 0.22108895 0.23247898 0.15424311 0.16531996 0.15947858 0.15691047
+ 0.15553006 0.15244881 0.17415222 0.19530395 0.15835334 0.15443013
+ 0.17730333 0.15253416 0.15255277 0.17044328 0.17223437 0.18623058
+ 0.21492836 0.15873511 0.32056993 0.18463367 0.15604755 0.20894248
+ 0.21239368 0.1650836  0.1535825  0.18891093 0.16862231 0.17614232
+ 0.15242051 0.17614232 0.32537736 0.15908675 0.15602061 0.284149
+ 0.18074179 0.65922132 0.17210558 0.16472687 0.15430244 0.1653026
+ 0.28911957 0.18122368 0.1535312  0.15793244 0.1784457  0.16406688
+ 0.15603269 0.15246975 0.16013835]</t>
+  </si>
+  <si>
+    <t>[0.19059254 0.2105817  0.17971614 0.17215635 0.18863854 0.18480222
+ 0.18939522 0.2662883  0.1900678  0.26744825 0.18600847 0.1731169
+ 0.22064914 0.21536575 0.18627836 0.21711026 0.2254367  0.17083155
+ 0.21373971 0.2214611  0.17220183 0.21571346 0.33075866 0.24388409
+ 0.36580575 0.17105044 0.18193014 0.22207129 0.18495627 0.17209812
+ 0.21824154 0.1935629  0.29762152 0.18522613 0.2907876  0.17129812
+ 0.2531513  0.2053309  0.314415   0.18151271 0.19426112 0.19098948
+ 0.19855936 0.20980856 0.17582984 0.20907523 0.19737464 0.23048098
+ 0.3569757  0.17644927 0.17067425 0.40712425 0.17170742 0.52101934
+ 0.27556655 0.21875225 0.21875225 0.3778064  0.20287035 0.1744032
+ 0.83671546 0.42535102 0.46553838 0.21675369 0.27882704 0.21797034
+ 0.20440696 0.17282064 0.40777218 0.17089985 0.19557257 0.2194078
+ 0.2105817  0.3330082  0.17075072 0.17060398 0.17754592 0.206235
+ 0.30832884 0.22306015 0.1988127  0.27261558 0.18399125 0.1799039
+ 0.24386175 0.34447575 0.17139784 0.20566419 0.20667839 0.20703554
+ 0.3375635  0.63424    0.21144538 0.17176038 0.17063893 0.20919845
+ 0.21214962 0.17211117 0.20440696 0.41260922 0.29356515 0.37184125
+ 0.37311476 0.19331834 0.3103345  0.18301435 0.29226092 0.20891789
+ 0.26066753 0.4239208  0.17909949 0.27371702]</t>
   </si>
 </sst>
 </file>
@@ -592,49 +600,49 @@
     </row>
     <row r="2" spans="1:25">
       <c r="A2">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="B2">
-        <v>0.186046511627907</v>
+        <v>0.2072072072072072</v>
       </c>
       <c r="C2">
-        <v>0.1798604875802994</v>
+        <v>0.182037279009819</v>
       </c>
       <c r="D2">
-        <v>0.1514332071389941</v>
+        <v>0.1642723804885967</v>
       </c>
       <c r="E2">
-        <v>-0.1877215769141913</v>
+        <v>-0.1081429420355633</v>
       </c>
       <c r="F2">
-        <v>0.5453473654473592</v>
+        <v>0.5522574300656523</v>
       </c>
       <c r="G2">
-        <v>0.1473963804716288</v>
+        <v>0.1629421042429434</v>
       </c>
       <c r="H2">
-        <v>0.6024927496910095</v>
+        <v>0.2224995869657268</v>
       </c>
       <c r="I2">
-        <v>0.03976028699846644</v>
+        <v>0.02843159650397472</v>
       </c>
       <c r="J2">
-        <v>0.01149132527544756</v>
+        <v>0.01150468682186103</v>
       </c>
       <c r="K2">
-        <v>0.1514332071389941</v>
+        <v>0.1642723804885967</v>
       </c>
       <c r="L2">
-        <v>0.4883928571428572</v>
+        <v>0.6314229249011858</v>
       </c>
       <c r="M2">
-        <v>0.2368373960711168</v>
+        <v>0.3885080504653821</v>
       </c>
       <c r="N2">
-        <v>0.2081525027751923</v>
+        <v>0.22571662068367</v>
       </c>
       <c r="O2">
-        <v>0.1017672792077065</v>
+        <v>0.08366741240024567</v>
       </c>
       <c r="P2">
         <v>10</v>
@@ -657,49 +665,49 @@
     </row>
     <row r="3" spans="1:25">
       <c r="A3">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="B3">
-        <v>0.186046511627907</v>
+        <v>0.2072072072072072</v>
       </c>
       <c r="C3">
-        <v>0.1514178768149055</v>
+        <v>0.1536805413966391</v>
       </c>
       <c r="D3">
-        <v>0.1514332071389941</v>
+        <v>0.1642723804885967</v>
       </c>
       <c r="E3">
-        <v>0.0001012348901420212</v>
+        <v>0.06447729716008377</v>
       </c>
       <c r="F3">
-        <v>0.4803941705700432</v>
+        <v>0.4831473412589758</v>
       </c>
       <c r="G3">
-        <v>3.314081304325867E-05</v>
+        <v>0.01529217963729989</v>
       </c>
       <c r="H3">
-        <v>3.314081304325867E-05</v>
+        <v>0.4001629183324106</v>
       </c>
       <c r="I3">
-        <v>1.098313489168224E-09</v>
+        <v>0.002418614043514911</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>0.01183213536542475</v>
       </c>
       <c r="K3">
-        <v>0.1514332071389941</v>
+        <v>0.1642723804885967</v>
       </c>
       <c r="L3">
-        <v>0.4883928571428572</v>
+        <v>0.6457509881422925</v>
       </c>
       <c r="M3">
-        <v>0.2368373960711168</v>
+        <v>0.3921651403426603</v>
       </c>
       <c r="N3">
-        <v>0.151404416104389</v>
+        <v>0.1533728656577426</v>
       </c>
       <c r="O3">
-        <v>0.002824993551611581</v>
+        <v>0.1044125530703763</v>
       </c>
       <c r="P3">
         <v>10</v>
@@ -728,49 +736,49 @@
     </row>
     <row r="4" spans="1:25">
       <c r="A4">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="B4">
-        <v>0.2298850574712644</v>
+        <v>0.2053571428571428</v>
       </c>
       <c r="C4">
-        <v>0.1887704879045486</v>
+        <v>0.1849401742219925</v>
       </c>
       <c r="D4">
-        <v>0.1770379178226979</v>
+        <v>0.1631855867346939</v>
       </c>
       <c r="E4">
-        <v>-0.06627150966382733</v>
+        <v>-0.1333119420814235</v>
       </c>
       <c r="F4">
-        <v>0.5632907745924173</v>
+        <v>0.5581014120604715</v>
       </c>
       <c r="G4">
-        <v>0.1377524738681728</v>
+        <v>0.1782246817435537</v>
       </c>
       <c r="H4">
-        <v>0.2984046737353007</v>
+        <v>0.3460728526115417</v>
       </c>
       <c r="I4">
-        <v>0.0231287553471751</v>
+        <v>0.03530949443239335</v>
       </c>
       <c r="J4">
-        <v>0.01398637907594219</v>
+        <v>0.01239738683935113</v>
       </c>
       <c r="K4">
-        <v>0.1770379178226979</v>
+        <v>0.1631855867346939</v>
       </c>
       <c r="L4">
-        <v>0.6235074626865671</v>
+        <v>0.5981924767953102</v>
       </c>
       <c r="M4">
-        <v>0.3861401364000659</v>
+        <v>0.3397146348841327</v>
       </c>
       <c r="N4">
-        <v>0.2144492566585541</v>
+        <v>0.222618505358696</v>
       </c>
       <c r="O4">
-        <v>0.1283896863460541</v>
+        <v>0.0903911367058754</v>
       </c>
       <c r="P4">
         <v>10</v>
@@ -793,49 +801,49 @@
     </row>
     <row r="5" spans="1:25">
       <c r="A5">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="B5">
-        <v>0.2298850574712644</v>
+        <v>0.2053571428571428</v>
       </c>
       <c r="C5">
-        <v>0.1692626029253006</v>
+        <v>0.1592216044664383</v>
       </c>
       <c r="D5">
-        <v>0.1770379178226979</v>
+        <v>0.1631855867346939</v>
       </c>
       <c r="E5">
-        <v>0.04391892422268651</v>
+        <v>0.02429125235612994</v>
       </c>
       <c r="F5">
-        <v>0.5195753954064737</v>
+        <v>0.4963798564145315</v>
       </c>
       <c r="G5">
-        <v>0.02584437991695843</v>
+        <v>0.05078752791242939</v>
       </c>
       <c r="H5">
-        <v>0.4574229121208191</v>
+        <v>0.6342399716377258</v>
       </c>
       <c r="I5">
-        <v>0.003421097226380759</v>
+        <v>0.00829098160200562</v>
       </c>
       <c r="J5">
-        <v>0.01435003099687999</v>
+        <v>0.01229057293207138</v>
       </c>
       <c r="K5">
-        <v>0.1770379178226979</v>
+        <v>0.1631855867346939</v>
       </c>
       <c r="L5">
-        <v>0.6235074626865671</v>
+        <v>0.6196873473375673</v>
       </c>
       <c r="M5">
-        <v>0.3861401364000659</v>
+        <v>0.3443963212886268</v>
       </c>
       <c r="N5">
-        <v>0.1772233098745346</v>
+        <v>0.1748965531587601</v>
       </c>
       <c r="O5">
-        <v>0.08502446115016937</v>
+        <v>0.1005334407091141</v>
       </c>
       <c r="P5">
         <v>10</v>

</xml_diff>